<commit_message>
changes as of 10th sep
</commit_message>
<xml_diff>
--- a/employee_input.xlsx
+++ b/employee_input.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pwcindia-my.sharepoint.com/personal/abhinandan_roy_pwc_com/Documents/Documents/work-in-sync/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pwcindia-my.sharepoint.com/personal/abhinandan_roy_pwc_com/Documents/work-in-sync/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="65" documentId="8_{2480ABF1-70E0-4400-B164-214693FD6CD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C202E1B8-48BA-4D89-BC56-15BF11539271}"/>
+  <xr:revisionPtr revIDLastSave="68" documentId="8_{2480ABF1-70E0-4400-B164-214693FD6CD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{87332863-1F17-4233-AB5A-6E99774796D0}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{887FC20F-A5A9-424F-A0B9-DA167AEAA032}"/>
   </bookViews>
@@ -170,7 +170,7 @@
     <t>Gourab Das</t>
   </si>
   <si>
-    <t>Tushti Thakur</t>
+    <t>Pankaj Devidas Bhagwat</t>
   </si>
 </sst>
 </file>
@@ -283,10 +283,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -951,7 +947,7 @@
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" s="3">
-        <v>101676413</v>
+        <v>101756438</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>43</v>

</xml_diff>